<commit_message>
Resolve work item W-001
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -471,7 +471,7 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>Ongoing</t>
+          <t>Resolved</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
@@ -491,10 +491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>需要找PM
-一樣的狀況
-所以....
-可以嗎???</t>
+          <t>需要找PM</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">

</xml_diff>

<commit_message>
Add new work item W-003 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,6 +554,45 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>System_FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>W-003</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>TS2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>新增一個測試</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AOT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new work item W-004 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,7 +583,11 @@
           <t>新增一個測試</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>2026-09-24</t>
@@ -595,6 +599,45 @@
         </is>
       </c>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>W-004</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TS2</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>ttttttttttt</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>AOT</t>
         </is>

</xml_diff>

<commit_message>
Add new work item W-005 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I5"/>
+  <dimension ref="A1:I6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -630,16 +630,63 @@
           <t>只是測試而已</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="G5" t="inlineStr">
         <is>
           <t>2026-09-24</t>
         </is>
       </c>
-      <c r="H5" t="inlineStr"/>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="I5" t="inlineStr">
         <is>
           <t>AOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>W-005</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>TS2</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>44</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>請夜班幫幫忙</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr"/>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="H6" t="inlineStr"/>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>SYSTEM_FT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update work item W-004
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -491,7 +491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>無資料測試一下</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
@@ -501,7 +501,7 @@
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>無資料</t>
+          <t>Kim</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">

</xml_diff>

<commit_message>
Add new work item W-006 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -554,6 +554,45 @@
       <c r="I3" t="inlineStr">
         <is>
           <t>MGMT_JTAG</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>W-006</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>AOT FAIL，需要幫忙追一下</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr"/>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr"/>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>AOT</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add new work item W-007 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:I5"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -583,14 +583,61 @@
           <t>AOT FAIL，需要幫忙追一下</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="G4" t="inlineStr">
         <is>
           <t>2026-09-27</t>
         </is>
       </c>
-      <c r="H4" t="inlineStr"/>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="I4" t="inlineStr">
+        <is>
+          <t>AOT</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>W-007</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>TS3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>TTEST</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr"/>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>2026-09-27</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr"/>
+      <c r="I5" t="inlineStr">
         <is>
           <t>AOT</t>
         </is>

</xml_diff>

<commit_message>
Add new work item W-008 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I7"/>
+  <dimension ref="A1:I8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -724,14 +724,61 @@
           <t>COU 100 —&gt; 離型紙未移除</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="G7" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="H7" t="inlineStr"/>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="I7" t="inlineStr">
+        <is>
+          <t>MGMT_FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>W-008</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>TS3</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>CPU 100度 —》離型紙未移除</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr"/>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H8" t="inlineStr"/>
+      <c r="I8" t="inlineStr">
         <is>
           <t>MGMT_FT</t>
         </is>

</xml_diff>

<commit_message>
Add new work item W-009 via Streamlit
</commit_message>
<xml_diff>
--- a/Work_item.xlsx
+++ b/Work_item.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -771,16 +771,63 @@
           <t>CPU 100度 —》離型紙未移除</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="G8" t="inlineStr">
         <is>
           <t>2026-10-02</t>
         </is>
       </c>
-      <c r="H8" t="inlineStr"/>
+      <c r="H8" t="inlineStr">
+        <is>
+          <t>無資料</t>
+        </is>
+      </c>
       <c r="I8" t="inlineStr">
         <is>
           <t>MGMT_FT</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>W-009</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>Ongoing</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>TS3</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>14</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>CPU 100度 —》離型紙未移除</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr"/>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="H9" t="inlineStr"/>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>MGMT_JTAG</t>
         </is>
       </c>
     </row>

</xml_diff>